<commit_message>
Interfaces template: Clock_1Hz + PNC_I_SORTER-<index> SORTER RUNNING (user 2026-10-18)
The MachineInterfaces template's two misnamed tags corrected (only xl/sharedStrings.xml changed):
- the clock "Clock 1Hz" -> TIA's "Clock_1Hz" (SORTER!P2, FVTGENERIC!P21)
- the sorter feedback "PNC_I_SORTER-<index> SORTER- RUNNING" -> "... SORTER RUNNING" (SORTER!O8),
  the name 07 Speed Control always read; 08 Gate Manager (TT01 + the door rows) now reads it too,
  through one helper (_sorter_running).

Parity: the frozen PL4 reference keeps the old spellings - read as the new on both sides, counted
(26), interface_elements uids re-stamped from the old spelling. Gate 76/76 + parity OK.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Shared/Templates/MachineInterfaces/TEMPLATE_INTERFACES_v0.0.xlsx
+++ b/Shared/Templates/MachineInterfaces/TEMPLATE_INTERFACES_v0.0.xlsx
@@ -133,7 +133,7 @@
     <t>Expression Side 1</t>
   </si>
   <si>
-    <t>"Clock 1Hz"</t>
+    <t>"Clock_1Hz"</t>
   </si>
   <si>
     <t>AREA</t>
@@ -190,7 +190,7 @@
     <t>PNC_Q_SORTER-&lt;index&gt; SAFETY ENCODER FAILURE</t>
   </si>
   <si>
-    <t>PNC_I_SORTER-&lt;index&gt; SORTER- RUNNING</t>
+    <t>PNC_I_SORTER-&lt;index&gt; SORTER RUNNING</t>
   </si>
   <si>
     <t>PNC_I_SORTER-&lt;index&gt; EMERGENCY RESET</t>

</xml_diff>